<commit_message>
scan: seg3 2026-06-22 22:40 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq4_2026-06-22.xlsx
+++ b/output/full_scan/batch_seq4_2026-06-22.xlsx
@@ -792,21 +792,21 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>3481</v>
+        <v>3707</v>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>群創</t>
+          <t>漢磊</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
         <v/>
       </c>
       <c r="D7" s="2" t="n">
-        <v>1140.196687668196</v>
+        <v>1130.443434956657</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>66</v>
+        <v>91.5</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
@@ -817,49 +817,49 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>72.26168150955721</v>
+        <v>64.42071255993068</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>37.45602884507969</v>
+        <v>30.76493603777575</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>1.746106408141673</v>
+        <v>1.477174189972248</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L7" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M7" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>0.7748167574596554</v>
+        <v>0.4573230841525006</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, volume_break, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, invest_trust_buy_2d, breakout_volume_confirm, mfi_strong, above_ichimoku_cloud</t>
+          <t>macd_golden_cross, above_ema60, ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, hist_turn_positive, adx_trending, stronger_than_market, obv_uptrend, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>3707</v>
+        <v>3481</v>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>漢磊</t>
+          <t>群創</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
         <v/>
       </c>
       <c r="D8" s="2" t="n">
-        <v>1130.443434956657</v>
+        <v>1130.196687668196</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>91.5</v>
+        <v>66</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
@@ -870,29 +870,29 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>64.42071255993068</v>
+        <v>72.26168150955721</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>30.76493603777575</v>
+        <v>37.45602884507969</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>1.477174189972248</v>
+        <v>1.746106408141673</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L8" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M8" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>0.4573230841525006</v>
+        <v>0.7748167574596554</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, above_ema60, ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, hist_turn_positive, adx_trending, stronger_than_market, obv_uptrend, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, volume_break, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, invest_trust_buy_2d, breakout_volume_confirm, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -1015,7 +1015,7 @@
         <v/>
       </c>
       <c r="D11" s="2" t="n">
-        <v>1071.839158962671</v>
+        <v>1081.839158962671</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>73.40000000000001</v>
@@ -1121,7 +1121,7 @@
         <v/>
       </c>
       <c r="D13" s="2" t="n">
-        <v>1039.859686656685</v>
+        <v>1049.859686656685</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>66.3</v>
@@ -1174,7 +1174,7 @@
         <v/>
       </c>
       <c r="D14" s="2" t="n">
-        <v>1020.213270207834</v>
+        <v>1010.213270207834</v>
       </c>
       <c r="E14" s="2" t="n">
         <v>42.7</v>
@@ -1216,21 +1216,21 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>3438</v>
+        <v>3714</v>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>類比科</t>
+          <t>富采</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
         <v/>
       </c>
       <c r="D15" s="2" t="n">
-        <v>1002.807051304218</v>
+        <v>1005.880039920602</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>78.5</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1241,16 +1241,16 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>64.44530268871236</v>
+        <v>57.65390115394436</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>34.15414062267372</v>
+        <v>16.63122874135879</v>
       </c>
       <c r="J15" s="2" t="n">
-        <v>1.816094749211985</v>
+        <v>1.199380797299028</v>
       </c>
       <c r="K15" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L15" s="2" t="n">
         <v>0</v>
@@ -1259,31 +1259,31 @@
         <v>-1</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>-0.1115767941520395</v>
+        <v>0.0720473341523869</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, liquidity_ok, foreign_buy_3d, adx_trending, stronger_than_market, obv_uptrend, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
+          <t>macd_golden_cross, above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, hist_turn_positive, foreign_buy_3d, stronger_than_market, obv_uptrend, dealer_buy_3d, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>3714</v>
+        <v>3438</v>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>富采</t>
+          <t>類比科</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
         <v/>
       </c>
       <c r="D16" s="2" t="n">
-        <v>995.8800399206024</v>
+        <v>1002.807051304218</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>72.90000000000001</v>
+        <v>78.5</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
@@ -1294,16 +1294,16 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>57.65390115394436</v>
+        <v>64.44530268871236</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>16.63122874135879</v>
+        <v>34.15414062267372</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>1.199380797299028</v>
+        <v>1.816094749211985</v>
       </c>
       <c r="K16" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L16" s="2" t="n">
         <v>0</v>
@@ -1312,11 +1312,11 @@
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>0.0720473341523869</v>
+        <v>-0.1115767941520395</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, hist_turn_positive, foreign_buy_3d, stronger_than_market, obv_uptrend, dealer_buy_3d, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, liquidity_ok, foreign_buy_3d, adx_trending, stronger_than_market, obv_uptrend, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -1598,7 +1598,7 @@
         <v/>
       </c>
       <c r="D22" s="2" t="n">
-        <v>944.1102164069476</v>
+        <v>924.1102164069476</v>
       </c>
       <c r="E22" s="2" t="n">
         <v>557</v>
@@ -1757,7 +1757,7 @@
         <v/>
       </c>
       <c r="D25" s="2" t="n">
-        <v>892.9615164259927</v>
+        <v>902.9615164259928</v>
       </c>
       <c r="E25" s="2" t="n">
         <v>25.95</v>
@@ -1905,21 +1905,21 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>3550</v>
+        <v>3680</v>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>聯穎</t>
+          <t>家登</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
         <v/>
       </c>
       <c r="D28" s="2" t="n">
-        <v>881.6359117223723</v>
+        <v>880.3919400611363</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>35.9</v>
+        <v>547</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
@@ -1930,13 +1930,13 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>78.63291082448265</v>
+        <v>56.04960404766393</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>45.71219348478207</v>
+        <v>13.15869168788597</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>2.487102058066101</v>
+        <v>1.258995562055865</v>
       </c>
       <c r="K28" s="2" t="n">
         <v>0</v>
@@ -1948,31 +1948,31 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>1.246118268079345</v>
+        <v>0.8723614778829152</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>macd_golden_cross, above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, hist_turn_positive, stronger_than_market, obv_uptrend, dealer_buy_3d, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>3680</v>
+        <v>3624</v>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>家登</t>
+          <t>光頡</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
         <v/>
       </c>
       <c r="D29" s="2" t="n">
-        <v>880.3919400611363</v>
+        <v>875.888469222643</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>547</v>
+        <v>176.5</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
@@ -1983,49 +1983,49 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>56.04960404766393</v>
+        <v>85.20631500498348</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>13.15869168788597</v>
+        <v>34.42488886193586</v>
       </c>
       <c r="J29" s="2" t="n">
-        <v>1.258995562055865</v>
+        <v>0.991309185296215</v>
       </c>
       <c r="K29" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L29" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M29" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>0.8723614778829152</v>
+        <v>4.91164437194525</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, hist_turn_positive, stronger_than_market, obv_uptrend, dealer_buy_3d, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, dealer_buy_3d, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>3624</v>
+        <v>3141</v>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>光頡</t>
+          <t>晶宏</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
         <v/>
       </c>
       <c r="D30" s="2" t="n">
-        <v>875.888469222643</v>
+        <v>873.5068525213269</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>176.5</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
@@ -2036,49 +2036,49 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>85.20631500498348</v>
+        <v>66.18020168353873</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>34.42488886193586</v>
+        <v>32.43403481191611</v>
       </c>
       <c r="J30" s="2" t="n">
-        <v>0.991309185296215</v>
+        <v>0.8014751722437315</v>
       </c>
       <c r="K30" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L30" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M30" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>4.91164437194525</v>
+        <v>-0.7937921305451434</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, dealer_buy_3d, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, foreign_buy_3d, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>3141</v>
+        <v>3406</v>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>晶宏</t>
+          <t>玉晶光</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
         <v/>
       </c>
       <c r="D31" s="2" t="n">
-        <v>873.5068525213269</v>
+        <v>872.2891076671208</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>78.40000000000001</v>
+        <v>774</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
@@ -2089,16 +2089,16 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>66.18020168353873</v>
+        <v>69.52995858008583</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>32.43403481191611</v>
+        <v>46.50786972908282</v>
       </c>
       <c r="J31" s="2" t="n">
-        <v>0.8014751722437315</v>
+        <v>1.328910766712084</v>
       </c>
       <c r="K31" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L31" s="2" t="n">
         <v>0</v>
@@ -2107,31 +2107,31 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>-0.7937921305451434</v>
+        <v>7.844677195767453</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, foreign_buy_3d, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>3675</v>
+        <v>3550</v>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>德微</t>
+          <t>聯穎</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
         <v/>
       </c>
       <c r="D32" s="2" t="n">
-        <v>867.2964267864029</v>
+        <v>871.6359117223723</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>405</v>
+        <v>35.9</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
@@ -2142,13 +2142,13 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>68.19634419053942</v>
+        <v>78.63291082448265</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>31.17821984438537</v>
+        <v>45.71219348478207</v>
       </c>
       <c r="J32" s="2" t="n">
-        <v>0.2968310550875776</v>
+        <v>2.487102058066101</v>
       </c>
       <c r="K32" s="2" t="n">
         <v>0</v>
@@ -2160,31 +2160,31 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>-0.1425584684760679</v>
+        <v>1.246118268079345</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, dealer_buy_3d, cci_momentum, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>3527</v>
+        <v>3675</v>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>聚積</t>
+          <t>德微</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
         <v/>
       </c>
       <c r="D33" s="2" t="n">
-        <v>863.4766944911818</v>
+        <v>867.2964267864029</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>70.2</v>
+        <v>405</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
@@ -2195,16 +2195,16 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>67.27928118127737</v>
+        <v>68.19634419053942</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>32.45451266622661</v>
+        <v>31.17821984438537</v>
       </c>
       <c r="J33" s="2" t="n">
-        <v>1.602511263887109</v>
+        <v>0.2968310550875776</v>
       </c>
       <c r="K33" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L33" s="2" t="n">
         <v>0</v>
@@ -2213,31 +2213,31 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>1.302181466542013</v>
+        <v>-0.1425584684760679</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, dealer_buy_3d, cci_momentum, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>3131</v>
+        <v>3311</v>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>弘塑</t>
+          <t>閎暉</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
         <v/>
       </c>
       <c r="D34" s="2" t="n">
-        <v>861.4059292823422</v>
+        <v>865.0399591686909</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>3585</v>
+        <v>40.25</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
@@ -2248,49 +2248,49 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>63.31918418701444</v>
+        <v>61.84534186720546</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>18.82090013214684</v>
+        <v>31.30046885245265</v>
       </c>
       <c r="J34" s="2" t="n">
-        <v>1.325108987708389</v>
+        <v>0.9699737906504888</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L34" s="2" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="M34" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>31.28883214927182</v>
+        <v>-0.0225263760473348</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, stronger_than_market, obv_uptrend, invest_trust_buy_2d, dealer_buy_3d, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, foreign_buy_3d, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>3265</v>
+        <v>3527</v>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>台星科</t>
+          <t>聚積</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
         <v/>
       </c>
       <c r="D35" s="2" t="n">
-        <v>857.9307725578986</v>
+        <v>863.4766944911818</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>193.5</v>
+        <v>70.2</v>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
@@ -2301,13 +2301,13 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>60.27477866480992</v>
+        <v>67.27928118127737</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>16.65809824073256</v>
+        <v>32.45451266622661</v>
       </c>
       <c r="J35" s="2" t="n">
-        <v>1.233678428956675</v>
+        <v>1.602511263887109</v>
       </c>
       <c r="K35" s="2" t="n">
         <v>2</v>
@@ -2319,31 +2319,31 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>0.4630977843997376</v>
+        <v>1.302181466542013</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, above_ema60, ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, hist_turn_positive, obv_uptrend, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>3406</v>
+        <v>3131</v>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>玉晶光</t>
+          <t>弘塑</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
         <v/>
       </c>
       <c r="D36" s="2" t="n">
-        <v>857.2891076671208</v>
+        <v>861.4059292823422</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>774</v>
+        <v>3585</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
@@ -2354,49 +2354,49 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>69.52995858008583</v>
+        <v>63.31918418701444</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>46.50786972908282</v>
+        <v>18.82090013214684</v>
       </c>
       <c r="J36" s="2" t="n">
-        <v>1.328910766712084</v>
+        <v>1.325108987708389</v>
       </c>
       <c r="K36" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L36" s="2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="M36" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>7.844677195767453</v>
+        <v>31.28883214927182</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, stronger_than_market, obv_uptrend, invest_trust_buy_2d, dealer_buy_3d, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>3311</v>
+        <v>3265</v>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>閎暉</t>
+          <t>台星科</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
         <v/>
       </c>
       <c r="D37" s="2" t="n">
-        <v>855.0399591686909</v>
+        <v>857.9307725578986</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>40.25</v>
+        <v>193.5</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
@@ -2407,16 +2407,16 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>61.84534186720546</v>
+        <v>60.27477866480992</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>31.30046885245265</v>
+        <v>16.65809824073256</v>
       </c>
       <c r="J37" s="2" t="n">
-        <v>0.9699737906504888</v>
+        <v>1.233678428956675</v>
       </c>
       <c r="K37" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L37" s="2" t="n">
         <v>0</v>
@@ -2425,11 +2425,11 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>-0.0225263760473348</v>
+        <v>0.4630977843997376</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, foreign_buy_3d, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>macd_golden_cross, above_ema60, ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, hist_turn_positive, obv_uptrend, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -2806,21 +2806,21 @@
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>3303</v>
+        <v>3592</v>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>岱稜</t>
+          <t>瑞鼎</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
         <v/>
       </c>
       <c r="D45" s="2" t="n">
-        <v>807.8357311824307</v>
+        <v>808.0638924730956</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>60.2</v>
+        <v>285</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
@@ -2831,49 +2831,49 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>68.57541127075211</v>
+        <v>60.75288678003712</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>34.004015715644</v>
+        <v>17.15383392431712</v>
       </c>
       <c r="J45" s="2" t="n">
-        <v>1.083573118243061</v>
+        <v>1.886675863216412</v>
       </c>
       <c r="K45" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L45" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M45" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>0.951981236432685</v>
+        <v>-0.1096970016281604</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, dealer_buy_3d, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>3455</v>
+        <v>3303</v>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>由田</t>
+          <t>岱稜</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
         <v/>
       </c>
       <c r="D46" s="2" t="n">
-        <v>805.4848372694787</v>
+        <v>807.8357311824307</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>266</v>
+        <v>60.2</v>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
@@ -2884,16 +2884,16 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>60.33006093555528</v>
+        <v>68.57541127075211</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>21.49855963408047</v>
+        <v>34.004015715644</v>
       </c>
       <c r="J46" s="2" t="n">
-        <v>1.789253493273612</v>
+        <v>1.083573118243061</v>
       </c>
       <c r="K46" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L46" s="2" t="n">
         <v>0</v>
@@ -2902,31 +2902,31 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>2.627966093965738</v>
+        <v>0.951981236432685</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, dealer_buy_3d, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>3484</v>
+        <v>3455</v>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>崧騰</t>
+          <t>由田</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
         <v/>
       </c>
       <c r="D47" s="2" t="n">
-        <v>805.1083271412338</v>
+        <v>805.4848372694787</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>52.9</v>
+        <v>266</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
@@ -2937,16 +2937,16 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>71.68317818250299</v>
+        <v>60.33006093555528</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>24.77508467262347</v>
+        <v>21.49855963408047</v>
       </c>
       <c r="J47" s="2" t="n">
-        <v>6.829940482745084</v>
+        <v>1.789253493273612</v>
       </c>
       <c r="K47" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L47" s="2" t="n">
         <v>0</v>
@@ -2955,31 +2955,31 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>1.042099753375455</v>
+        <v>2.627966093965738</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, volume_break, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>3592</v>
+        <v>3484</v>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>瑞鼎</t>
+          <t>崧騰</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
         <v/>
       </c>
       <c r="D48" s="2" t="n">
-        <v>798.0638924730956</v>
+        <v>805.1083271412338</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>285</v>
+        <v>52.9</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
@@ -2990,49 +2990,49 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>60.75288678003712</v>
+        <v>71.68317818250299</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>17.15383392431712</v>
+        <v>24.77508467262347</v>
       </c>
       <c r="J48" s="2" t="n">
-        <v>1.886675863216412</v>
+        <v>6.829940482745084</v>
       </c>
       <c r="K48" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L48" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M48" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>-0.1096970016281604</v>
+        <v>1.042099753375455</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, volume_break, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>3583</v>
+        <v>3630</v>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>辛耘</t>
+          <t>新鉅科</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
         <v/>
       </c>
       <c r="D49" s="2" t="n">
-        <v>785.5654076392259</v>
+        <v>781.2195563711762</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>889</v>
+        <v>33.65</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
@@ -3043,16 +3043,16 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>58.40190834356723</v>
+        <v>64.97140442488922</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>20.8756195180744</v>
+        <v>27.55255147073269</v>
       </c>
       <c r="J49" s="2" t="n">
-        <v>1.058456039761434</v>
+        <v>0.9219556371176162</v>
       </c>
       <c r="K49" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L49" s="2" t="n">
         <v>0</v>
@@ -3061,31 +3061,31 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>-0.37879956872783</v>
+        <v>0.6846685329886983</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>3630</v>
+        <v>3520</v>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>新鉅科</t>
+          <t>華盈</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
         <v/>
       </c>
       <c r="D50" s="2" t="n">
-        <v>781.2195563711762</v>
+        <v>778.3842363980134</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>33.65</v>
+        <v>16.8</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -3096,16 +3096,16 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>64.97140442488922</v>
+        <v>55.45464572885061</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>27.55255147073269</v>
+        <v>35.74806932414902</v>
       </c>
       <c r="J50" s="2" t="n">
-        <v>0.9219556371176162</v>
+        <v>0.4598568740232251</v>
       </c>
       <c r="K50" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L50" s="2" t="n">
         <v>0</v>
@@ -3114,31 +3114,31 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>0.6846685329886983</v>
+        <v>-0.011889840657288</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>3520</v>
+        <v>3465</v>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>華盈</t>
+          <t>進泰電子</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
         <v/>
       </c>
       <c r="D51" s="2" t="n">
-        <v>778.3842363980134</v>
+        <v>778.3015312809114</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>16.8</v>
+        <v>39.9</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
@@ -3149,16 +3149,16 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>55.45464572885061</v>
+        <v>73.62428770506888</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>35.74806932414902</v>
+        <v>36.99902776569249</v>
       </c>
       <c r="J51" s="2" t="n">
-        <v>0.4598568740232251</v>
+        <v>1.469229784296306</v>
       </c>
       <c r="K51" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L51" s="2" t="n">
         <v>0</v>
@@ -3167,31 +3167,31 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>-0.011889840657288</v>
+        <v>0.898974376034532</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, rsi_strong, breakout_20d, market_above_ma60, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>3465</v>
+        <v>3583</v>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>進泰電子</t>
+          <t>辛耘</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
         <v/>
       </c>
       <c r="D52" s="2" t="n">
-        <v>778.3015312809114</v>
+        <v>775.5654076392259</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>39.9</v>
+        <v>889</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
@@ -3202,13 +3202,13 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>73.62428770506888</v>
+        <v>58.40190834356723</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>36.99902776569249</v>
+        <v>20.8756195180744</v>
       </c>
       <c r="J52" s="2" t="n">
-        <v>1.469229784296306</v>
+        <v>1.058456039761434</v>
       </c>
       <c r="K52" s="2" t="n">
         <v>0</v>
@@ -3220,11 +3220,11 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>0.898974376034532</v>
+        <v>-0.37879956872783</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, rsi_strong, breakout_20d, market_above_ma60, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -3442,21 +3442,21 @@
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>3231</v>
+        <v>3706</v>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>緯創</t>
+          <t>神達</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
         <v/>
       </c>
       <c r="D57" s="2" t="n">
-        <v>736.8536157430791</v>
+        <v>739.8286150262622</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>162.5</v>
+        <v>87.40000000000001</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
@@ -3467,25 +3467,25 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>54.30936120980893</v>
+        <v>50.7911930199166</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>17.56622256745875</v>
+        <v>13.74389208776697</v>
       </c>
       <c r="J57" s="2" t="n">
-        <v>0.5934922803590745</v>
+        <v>0.6239148051126658</v>
       </c>
       <c r="K57" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L57" s="2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M57" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>-1.356785101922135</v>
+        <v>-0.6179857828160394</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
@@ -3495,21 +3495,21 @@
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>3227</v>
+        <v>3231</v>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>原相</t>
+          <t>緯創</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
         <v/>
       </c>
       <c r="D58" s="2" t="n">
-        <v>733.0584380214254</v>
+        <v>736.8536157430791</v>
       </c>
       <c r="E58" s="2" t="n">
-        <v>230</v>
+        <v>162.5</v>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
@@ -3520,49 +3520,49 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>58.54697432451807</v>
+        <v>54.30936120980893</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>22.29506266061848</v>
+        <v>17.56622256745875</v>
       </c>
       <c r="J58" s="2" t="n">
-        <v>1.886212681405242</v>
+        <v>0.5934922803590745</v>
       </c>
       <c r="K58" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L58" s="2" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="M58" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>-0.1753356500670888</v>
+        <v>-1.356785101922135</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, invest_trust_buy_2d, dealer_buy_3d, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>3362</v>
+        <v>3227</v>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>先進光</t>
+          <t>原相</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
         <v/>
       </c>
       <c r="D59" s="2" t="n">
-        <v>731.4920376993841</v>
+        <v>733.0584380214254</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>205</v>
+        <v>230</v>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
@@ -3573,49 +3573,49 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>77.50972727252383</v>
+        <v>58.54697432451807</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>44.41944908006825</v>
+        <v>22.29506266061848</v>
       </c>
       <c r="J59" s="2" t="n">
-        <v>0.9492037699384104</v>
+        <v>1.886212681405242</v>
       </c>
       <c r="K59" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="L59" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="L59" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="M59" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>6.509331853913302</v>
+        <v>-0.1753356500670888</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>3706</v>
+        <v>3362</v>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>神達</t>
+          <t>先進光</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
         <v/>
       </c>
       <c r="D60" s="2" t="n">
-        <v>724.8286150262622</v>
+        <v>731.4920376993841</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>87.40000000000001</v>
+        <v>205</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
@@ -3626,29 +3626,29 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>50.7911930199166</v>
+        <v>77.50972727252383</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>13.74389208776697</v>
+        <v>44.41944908006825</v>
       </c>
       <c r="J60" s="2" t="n">
-        <v>0.6239148051126658</v>
+        <v>0.9492037699384104</v>
       </c>
       <c r="K60" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L60" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M60" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>-0.6179857828160394</v>
+        <v>6.509331853913302</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, invest_trust_buy_2d, dealer_buy_3d, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -4237,21 +4237,21 @@
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>3673</v>
+        <v>3305</v>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>TPK-KY</t>
+          <t>昇貿</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
         <v/>
       </c>
       <c r="D72" s="2" t="n">
-        <v>671.5517330220783</v>
+        <v>667.8598628222554</v>
       </c>
       <c r="E72" s="2" t="n">
-        <v>88.5</v>
+        <v>147</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
@@ -4262,16 +4262,16 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>61.34263205151396</v>
+        <v>53.88197701809596</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>30.24548074961963</v>
+        <v>23.2288852919096</v>
       </c>
       <c r="J72" s="2" t="n">
-        <v>0.9672721619824138</v>
+        <v>0.5004286825871733</v>
       </c>
       <c r="K72" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L72" s="2" t="n">
         <v>0</v>
@@ -4280,11 +4280,11 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>-0.6974675990064316</v>
+        <v>-1.993182394565167</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, dealer_buy_3d, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -4502,21 +4502,21 @@
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>3305</v>
+        <v>3673</v>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>昇貿</t>
+          <t>TPK-KY</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
         <v/>
       </c>
       <c r="D77" s="2" t="n">
-        <v>657.8598628222554</v>
+        <v>656.5517330220783</v>
       </c>
       <c r="E77" s="2" t="n">
-        <v>147</v>
+        <v>88.5</v>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
@@ -4527,16 +4527,16 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>53.88197701809596</v>
+        <v>61.34263205151396</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>23.2288852919096</v>
+        <v>30.24548074961963</v>
       </c>
       <c r="J77" s="2" t="n">
-        <v>0.5004286825871733</v>
+        <v>0.9672721619824138</v>
       </c>
       <c r="K77" s="2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L77" s="2" t="n">
         <v>0</v>
@@ -4545,11 +4545,11 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>-1.993182394565167</v>
+        <v>-0.6974675990064316</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, dealer_buy_3d, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -5032,21 +5032,21 @@
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>3687</v>
+        <v>3704</v>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>歐買尬</t>
+          <t>合勤控</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
         <v/>
       </c>
       <c r="D87" s="2" t="n">
-        <v>613.2246935901871</v>
+        <v>614.005842275344</v>
       </c>
       <c r="E87" s="2" t="n">
-        <v>78</v>
+        <v>48.5</v>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
@@ -5057,16 +5057,16 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>59.34037107286859</v>
+        <v>61.77234382079236</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>30.49130489005564</v>
+        <v>34.8180965192699</v>
       </c>
       <c r="J87" s="2" t="n">
-        <v>0.8035665119112906</v>
+        <v>0.5307917408635052</v>
       </c>
       <c r="K87" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L87" s="2" t="n">
         <v>0</v>
@@ -5075,31 +5075,31 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>-0.0101622144645068</v>
+        <v>-0.2056783609273251</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>3529</v>
+        <v>3687</v>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>力旺</t>
+          <t>歐買尬</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
         <v/>
       </c>
       <c r="D88" s="2" t="n">
-        <v>613.0972710456424</v>
+        <v>613.2246935901871</v>
       </c>
       <c r="E88" s="2" t="n">
-        <v>3180</v>
+        <v>78</v>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
@@ -5110,49 +5110,49 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>43.77208415301688</v>
+        <v>59.34037107286859</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>22.59457454145671</v>
+        <v>30.49130489005564</v>
       </c>
       <c r="J88" s="2" t="n">
-        <v>0.6829393924406626</v>
+        <v>0.8035665119112906</v>
       </c>
       <c r="K88" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L88" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M88" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>1.70024473622307</v>
+        <v>-0.0101622144645068</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, hist_turn_positive, adx_trending, invest_trust_buy_2d</t>
+          <t>above_ema60, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>3704</v>
+        <v>3529</v>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>合勤控</t>
+          <t>力旺</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
         <v/>
       </c>
       <c r="D89" s="2" t="n">
-        <v>604.005842275344</v>
+        <v>613.0972710456424</v>
       </c>
       <c r="E89" s="2" t="n">
-        <v>48.5</v>
+        <v>3180</v>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
@@ -5163,29 +5163,29 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>61.77234382079236</v>
+        <v>43.77208415301688</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>34.8180965192699</v>
+        <v>22.59457454145671</v>
       </c>
       <c r="J89" s="2" t="n">
-        <v>0.5307917408635052</v>
+        <v>0.6829393924406626</v>
       </c>
       <c r="K89" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L89" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M89" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>-0.2056783609273251</v>
+        <v>1.70024473622307</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, above_ichimoku_cloud</t>
+          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, hist_turn_positive, adx_trending, invest_trust_buy_2d</t>
         </is>
       </c>
     </row>
@@ -5403,21 +5403,21 @@
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>3535</v>
+        <v>3716</v>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>晶彩科</t>
+          <t>中化控股</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
         <v/>
       </c>
       <c r="D94" s="2" t="n">
-        <v>575.3075720515491</v>
+        <v>574.2150384201967</v>
       </c>
       <c r="E94" s="2" t="n">
-        <v>128.5</v>
+        <v>34.65</v>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
@@ -5428,13 +5428,13 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>49.93924454687225</v>
+        <v>51.75048837762611</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>21.48660861444925</v>
+        <v>26.50182621681756</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>0.9566685319898171</v>
+        <v>0.6333354945597074</v>
       </c>
       <c r="K94" s="2" t="n">
         <v>0</v>
@@ -5446,31 +5446,31 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>0.0999533328780184</v>
+        <v>-0.0911583282182207</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>3716</v>
+        <v>3535</v>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>中化控股</t>
+          <t>晶彩科</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
         <v/>
       </c>
       <c r="D95" s="2" t="n">
-        <v>574.2150384201967</v>
+        <v>565.3075720515491</v>
       </c>
       <c r="E95" s="2" t="n">
-        <v>34.65</v>
+        <v>128.5</v>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
@@ -5481,13 +5481,13 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>51.75048837762611</v>
+        <v>49.93924454687225</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>26.50182621681756</v>
+        <v>21.48660861444925</v>
       </c>
       <c r="J95" s="2" t="n">
-        <v>0.6333354945597074</v>
+        <v>0.9566685319898171</v>
       </c>
       <c r="K95" s="2" t="n">
         <v>0</v>
@@ -5499,31 +5499,31 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>-0.0911583282182207</v>
+        <v>0.0999533328780184</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>3576</v>
+        <v>3485</v>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>聯合再生</t>
+          <t>敘豐</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>570.082146079221</v>
+        <v>560.9676459472147</v>
       </c>
       <c r="E96" s="2" t="n">
-        <v>18.05</v>
+        <v>319.5</v>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
@@ -5534,16 +5534,16 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>49.00828305495014</v>
+        <v>50.93952067125235</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>22.66382837381164</v>
+        <v>15.08510164229576</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>0.5326935002116774</v>
+        <v>0.699872054699514</v>
       </c>
       <c r="K96" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L96" s="2" t="n">
         <v>0</v>
@@ -5552,31 +5552,31 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>0.007192002870832</v>
+        <v>-3.854686863258451</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>3485</v>
+        <v>3628</v>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>敘豐</t>
+          <t>盈正</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
         <v/>
       </c>
       <c r="D97" s="2" t="n">
-        <v>560.9676459472147</v>
+        <v>556.4868513390937</v>
       </c>
       <c r="E97" s="2" t="n">
-        <v>319.5</v>
+        <v>75.7</v>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
@@ -5587,13 +5587,13 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>50.93952067125235</v>
+        <v>62.16723127340285</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>15.08510164229576</v>
+        <v>20.73866168268252</v>
       </c>
       <c r="J97" s="2" t="n">
-        <v>0.699872054699514</v>
+        <v>0.8536886664345359</v>
       </c>
       <c r="K97" s="2" t="n">
         <v>0</v>
@@ -5605,31 +5605,31 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>-3.854686863258451</v>
+        <v>0.2170926462761062</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
-        <v>3628</v>
+        <v>3576</v>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>盈正</t>
+          <t>聯合再生</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
         <v/>
       </c>
       <c r="D98" s="2" t="n">
-        <v>556.4868513390937</v>
+        <v>555.082146079221</v>
       </c>
       <c r="E98" s="2" t="n">
-        <v>75.7</v>
+        <v>18.05</v>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
@@ -5640,16 +5640,16 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>62.16723127340285</v>
+        <v>49.00828305495014</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>20.73866168268252</v>
+        <v>22.66382837381164</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>0.8536886664345359</v>
+        <v>0.5326935002116774</v>
       </c>
       <c r="K98" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L98" s="2" t="n">
         <v>0</v>
@@ -5658,11 +5658,11 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>0.2170926462761062</v>
+        <v>0.007192002870832</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
@@ -6357,21 +6357,21 @@
     </row>
     <row r="112">
       <c r="A112" s="2" t="n">
-        <v>3339</v>
+        <v>3694</v>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>泰谷</t>
+          <t>海華</t>
         </is>
       </c>
       <c r="C112" s="2" t="n">
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>518.821804164223</v>
+        <v>519.9125470989625</v>
       </c>
       <c r="E112" s="2" t="n">
-        <v>48.2</v>
+        <v>62</v>
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
@@ -6382,16 +6382,16 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>50.47543529039581</v>
+        <v>46.31765257631338</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>13.24783713183411</v>
+        <v>22.5457907993813</v>
       </c>
       <c r="J112" s="2" t="n">
-        <v>0.8344587325729846</v>
+        <v>1.00217363805531</v>
       </c>
       <c r="K112" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L112" s="2" t="n">
         <v>0</v>
@@ -6400,31 +6400,31 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>0.4837216901270664</v>
+        <v>-0.6414765886739584</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, liquidity_ok, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
-        <v>3533</v>
+        <v>3339</v>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>嘉澤</t>
+          <t>泰谷</t>
         </is>
       </c>
       <c r="C113" s="2" t="n">
         <v/>
       </c>
       <c r="D113" s="2" t="n">
-        <v>514.1720697366537</v>
+        <v>518.821804164223</v>
       </c>
       <c r="E113" s="2" t="n">
-        <v>2315</v>
+        <v>48.2</v>
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
@@ -6435,16 +6435,16 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>45.56583292183997</v>
+        <v>50.47543529039581</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>20.47655979658528</v>
+        <v>13.24783713183411</v>
       </c>
       <c r="J113" s="2" t="n">
-        <v>0.6167123724564944</v>
+        <v>0.8344587325729846</v>
       </c>
       <c r="K113" s="2" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L113" s="2" t="n">
         <v>0</v>
@@ -6453,31 +6453,31 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>-10.00377851411068</v>
+        <v>0.4837216901270664</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, dealer_buy_3d</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, liquidity_ok, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="n">
-        <v>3287</v>
+        <v>3533</v>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>廣寰科</t>
+          <t>嘉澤</t>
         </is>
       </c>
       <c r="C114" s="2" t="n">
         <v/>
       </c>
       <c r="D114" s="2" t="n">
-        <v>512.8739784481096</v>
+        <v>514.1720697366537</v>
       </c>
       <c r="E114" s="2" t="n">
-        <v>33.75</v>
+        <v>2315</v>
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
@@ -6488,16 +6488,16 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>49.82585191159364</v>
+        <v>45.56583292183997</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>22.1302407108494</v>
+        <v>20.47655979658528</v>
       </c>
       <c r="J114" s="2" t="n">
-        <v>0.2045152005819464</v>
+        <v>0.6167123724564944</v>
       </c>
       <c r="K114" s="2" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="L114" s="2" t="n">
         <v>0</v>
@@ -6506,31 +6506,31 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>-0.4486717116322813</v>
+        <v>-10.00377851411068</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, dealer_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="n">
-        <v>3694</v>
+        <v>3287</v>
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>海華</t>
+          <t>廣寰科</t>
         </is>
       </c>
       <c r="C115" s="2" t="n">
         <v/>
       </c>
       <c r="D115" s="2" t="n">
-        <v>509.9125470989625</v>
+        <v>512.8739784481096</v>
       </c>
       <c r="E115" s="2" t="n">
-        <v>62</v>
+        <v>33.75</v>
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
@@ -6541,16 +6541,16 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>46.31765257631338</v>
+        <v>49.82585191159364</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>22.5457907993813</v>
+        <v>22.1302407108494</v>
       </c>
       <c r="J115" s="2" t="n">
-        <v>1.00217363805531</v>
+        <v>0.2045152005819464</v>
       </c>
       <c r="K115" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L115" s="2" t="n">
         <v>0</v>
@@ -6559,11 +6559,11 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>-0.6414765886739584</v>
+        <v>-0.4486717116322813</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -6834,21 +6834,21 @@
     </row>
     <row r="121">
       <c r="A121" s="2" t="n">
-        <v>3596</v>
+        <v>3135</v>
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>智易</t>
+          <t>凌航</t>
         </is>
       </c>
       <c r="C121" s="2" t="n">
         <v/>
       </c>
       <c r="D121" s="2" t="n">
-        <v>497.6751988455001</v>
+        <v>493.9945230066066</v>
       </c>
       <c r="E121" s="2" t="n">
-        <v>188</v>
+        <v>207</v>
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
@@ -6859,49 +6859,49 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>52.60205051409029</v>
+        <v>51.78713153720336</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>20.83811708821046</v>
+        <v>23.05842628506039</v>
       </c>
       <c r="J121" s="2" t="n">
-        <v>1.049319449664037</v>
+        <v>0.734647657873297</v>
       </c>
       <c r="K121" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L121" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M121" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>-0.1078203106482407</v>
+        <v>-5.390761217192599</v>
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, dealer_buy_3d, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="n">
-        <v>3135</v>
+        <v>3596</v>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>凌航</t>
+          <t>智易</t>
         </is>
       </c>
       <c r="C122" s="2" t="n">
         <v/>
       </c>
       <c r="D122" s="2" t="n">
-        <v>478.9945230066066</v>
+        <v>487.6751988455001</v>
       </c>
       <c r="E122" s="2" t="n">
-        <v>207</v>
+        <v>188</v>
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
@@ -6912,29 +6912,29 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>51.78713153720336</v>
+        <v>52.60205051409029</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>23.05842628506039</v>
+        <v>20.83811708821046</v>
       </c>
       <c r="J122" s="2" t="n">
-        <v>0.734647657873297</v>
+        <v>1.049319449664037</v>
       </c>
       <c r="K122" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L122" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M122" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>-5.390761217192599</v>
+        <v>-0.1078203106482407</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, dealer_buy_3d, above_ichimoku_cloud</t>
+          <t>above_ema60, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -7629,21 +7629,21 @@
     </row>
     <row r="136">
       <c r="A136" s="2" t="n">
-        <v>3702</v>
+        <v>3594</v>
       </c>
       <c r="B136" s="2" t="inlineStr">
         <is>
-          <t>大聯大</t>
+          <t>磐儀</t>
         </is>
       </c>
       <c r="C136" s="2" t="n">
         <v/>
       </c>
       <c r="D136" s="2" t="n">
-        <v>437.6737515703883</v>
+        <v>436.4501157044615</v>
       </c>
       <c r="E136" s="2" t="n">
-        <v>112.5</v>
+        <v>48</v>
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
@@ -7654,49 +7654,49 @@
         <v>0</v>
       </c>
       <c r="H136" s="2" t="n">
-        <v>52.59748221158775</v>
+        <v>48.7665729197427</v>
       </c>
       <c r="I136" s="2" t="n">
-        <v>28.53854811019093</v>
+        <v>14.06044978876462</v>
       </c>
       <c r="J136" s="2" t="n">
-        <v>0.6059772293666649</v>
+        <v>0.8530255202134293</v>
       </c>
       <c r="K136" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L136" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M136" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N136" s="2" t="n">
-        <v>-0.8228878063050823</v>
+        <v>0.059573984566036</v>
       </c>
       <c r="O136" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
+          <t>macd_golden_cross, above_ema60, ema60_gt_ema120, market_above_ma60, hist_turn_positive, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="n">
-        <v>3594</v>
+        <v>3531</v>
       </c>
       <c r="B137" s="2" t="inlineStr">
         <is>
-          <t>磐儀</t>
+          <t>先益</t>
         </is>
       </c>
       <c r="C137" s="2" t="n">
         <v/>
       </c>
       <c r="D137" s="2" t="n">
-        <v>436.4501157044615</v>
+        <v>436.0423831938822</v>
       </c>
       <c r="E137" s="2" t="n">
-        <v>48</v>
+        <v>23.05</v>
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
@@ -7707,16 +7707,16 @@
         <v>0</v>
       </c>
       <c r="H137" s="2" t="n">
-        <v>48.7665729197427</v>
+        <v>51.76184407994224</v>
       </c>
       <c r="I137" s="2" t="n">
-        <v>14.06044978876462</v>
+        <v>8.566357027043663</v>
       </c>
       <c r="J137" s="2" t="n">
-        <v>0.8530255202134293</v>
+        <v>0.7685508972831726</v>
       </c>
       <c r="K137" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L137" s="2" t="n">
         <v>0</v>
@@ -7725,31 +7725,31 @@
         <v>-1</v>
       </c>
       <c r="N137" s="2" t="n">
-        <v>0.059573984566036</v>
+        <v>0.1058383182346062</v>
       </c>
       <c r="O137" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, above_ema60, ema60_gt_ema120, market_above_ma60, hist_turn_positive, obv_uptrend</t>
+          <t>macd_golden_cross, above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, hist_turn_positive, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="n">
-        <v>3531</v>
+        <v>3653</v>
       </c>
       <c r="B138" s="2" t="inlineStr">
         <is>
-          <t>先益</t>
+          <t>健策</t>
         </is>
       </c>
       <c r="C138" s="2" t="n">
         <v/>
       </c>
       <c r="D138" s="2" t="n">
-        <v>436.0423831938822</v>
+        <v>430.1338787044289</v>
       </c>
       <c r="E138" s="2" t="n">
-        <v>23.05</v>
+        <v>3840</v>
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
@@ -7760,16 +7760,16 @@
         <v>0</v>
       </c>
       <c r="H138" s="2" t="n">
-        <v>51.76184407994224</v>
+        <v>50.23712379772032</v>
       </c>
       <c r="I138" s="2" t="n">
-        <v>8.566357027043663</v>
+        <v>15.33793728776078</v>
       </c>
       <c r="J138" s="2" t="n">
-        <v>0.7685508972831726</v>
+        <v>0.7723170251738766</v>
       </c>
       <c r="K138" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L138" s="2" t="n">
         <v>0</v>
@@ -7778,31 +7778,31 @@
         <v>-1</v>
       </c>
       <c r="N138" s="2" t="n">
-        <v>0.1058383182346062</v>
+        <v>39.19596538187471</v>
       </c>
       <c r="O138" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, hist_turn_positive, obv_uptrend, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="n">
-        <v>3653</v>
+        <v>3332</v>
       </c>
       <c r="B139" s="2" t="inlineStr">
         <is>
-          <t>健策</t>
+          <t>幸康</t>
         </is>
       </c>
       <c r="C139" s="2" t="n">
         <v/>
       </c>
       <c r="D139" s="2" t="n">
-        <v>430.1338787044289</v>
+        <v>429.394652325315</v>
       </c>
       <c r="E139" s="2" t="n">
-        <v>3840</v>
+        <v>64.8</v>
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
@@ -7813,16 +7813,16 @@
         <v>0</v>
       </c>
       <c r="H139" s="2" t="n">
-        <v>50.23712379772032</v>
+        <v>50.1720612118065</v>
       </c>
       <c r="I139" s="2" t="n">
-        <v>15.33793728776078</v>
+        <v>32.05687782614656</v>
       </c>
       <c r="J139" s="2" t="n">
-        <v>0.7723170251738766</v>
+        <v>0.1382597219696227</v>
       </c>
       <c r="K139" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L139" s="2" t="n">
         <v>0</v>
@@ -7831,31 +7831,31 @@
         <v>-1</v>
       </c>
       <c r="N139" s="2" t="n">
-        <v>39.19596538187471</v>
+        <v>-0.2697245855413001</v>
       </c>
       <c r="O139" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="n">
-        <v>3332</v>
+        <v>3685</v>
       </c>
       <c r="B140" s="2" t="inlineStr">
         <is>
-          <t>幸康</t>
+          <t>元創精密</t>
         </is>
       </c>
       <c r="C140" s="2" t="n">
         <v/>
       </c>
       <c r="D140" s="2" t="n">
-        <v>429.394652325315</v>
+        <v>428.6524849038919</v>
       </c>
       <c r="E140" s="2" t="n">
-        <v>64.8</v>
+        <v>30.3</v>
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
@@ -7866,16 +7866,16 @@
         <v>0</v>
       </c>
       <c r="H140" s="2" t="n">
-        <v>50.1720612118065</v>
+        <v>55.20776589026109</v>
       </c>
       <c r="I140" s="2" t="n">
-        <v>32.05687782614656</v>
+        <v>10.89929141402712</v>
       </c>
       <c r="J140" s="2" t="n">
-        <v>0.1382597219696227</v>
+        <v>1.096061418320755</v>
       </c>
       <c r="K140" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L140" s="2" t="n">
         <v>0</v>
@@ -7884,31 +7884,31 @@
         <v>-1</v>
       </c>
       <c r="N140" s="2" t="n">
-        <v>-0.2697245855413001</v>
+        <v>0.3021544440643859</v>
       </c>
       <c r="O140" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, rsi_strong, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="n">
-        <v>3685</v>
+        <v>3702</v>
       </c>
       <c r="B141" s="2" t="inlineStr">
         <is>
-          <t>元創精密</t>
+          <t>大聯大</t>
         </is>
       </c>
       <c r="C141" s="2" t="n">
         <v/>
       </c>
       <c r="D141" s="2" t="n">
-        <v>428.6524849038919</v>
+        <v>427.6737515703883</v>
       </c>
       <c r="E141" s="2" t="n">
-        <v>30.3</v>
+        <v>112.5</v>
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
@@ -7919,29 +7919,29 @@
         <v>0</v>
       </c>
       <c r="H141" s="2" t="n">
-        <v>55.20776589026109</v>
+        <v>52.59748221158775</v>
       </c>
       <c r="I141" s="2" t="n">
-        <v>10.89929141402712</v>
+        <v>28.53854811019093</v>
       </c>
       <c r="J141" s="2" t="n">
-        <v>1.096061418320755</v>
+        <v>0.6059772293666649</v>
       </c>
       <c r="K141" s="2" t="n">
         <v>1</v>
       </c>
       <c r="L141" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M141" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N141" s="2" t="n">
-        <v>0.3021544440643859</v>
+        <v>-0.8228878063050823</v>
       </c>
       <c r="O141" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, rsi_strong, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>

</xml_diff>